<commit_message>
Add a origin rule from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/data/neslihan.xlsx
+++ b/cellstocks/data/neslihan.xlsx
@@ -368,6 +368,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -450,6 +455,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -619,6 +629,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -875,6 +890,11 @@
           <t xml:space="preserve">29.12.23</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -957,6 +977,11 @@
           <t xml:space="preserve">29.12.23</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -1039,6 +1064,11 @@
           <t xml:space="preserve">29.12.24</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -1556,6 +1586,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -1638,6 +1673,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -2242,6 +2282,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -2324,6 +2369,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -2406,6 +2456,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -2488,6 +2543,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -2570,6 +2630,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -2652,6 +2717,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -6015,6 +6085,11 @@
           <t xml:space="preserve">31.07.23</t>
         </is>
       </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L70" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -7454,6 +7529,11 @@
           <t xml:space="preserve">13.07.23</t>
         </is>
       </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L87" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -10290,6 +10370,11 @@
           <t xml:space="preserve">16.10.23</t>
         </is>
       </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L120" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -12194,6 +12279,11 @@
           <t xml:space="preserve">01.22.23</t>
         </is>
       </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L142" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -12276,6 +12366,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L143" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -12445,6 +12540,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L145" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -12614,6 +12714,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L147" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14001,6 +14106,11 @@
           <t xml:space="preserve">14.03.24</t>
         </is>
       </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L163" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14083,6 +14193,11 @@
           <t xml:space="preserve">14.03.24</t>
         </is>
       </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L164" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14165,6 +14280,11 @@
           <t xml:space="preserve">15.02.24</t>
         </is>
       </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L165" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14247,6 +14367,11 @@
           <t xml:space="preserve">14.03.24</t>
         </is>
       </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L166" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14329,6 +14454,11 @@
           <t xml:space="preserve">15.02.24</t>
         </is>
       </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L167" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14411,6 +14541,11 @@
           <t xml:space="preserve">14.03.24</t>
         </is>
       </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L168" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14493,6 +14628,11 @@
           <t xml:space="preserve">13.02.24</t>
         </is>
       </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L169" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14575,6 +14715,11 @@
           <t xml:space="preserve">14.03.24</t>
         </is>
       </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L170" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14657,6 +14802,11 @@
           <t xml:space="preserve">13.02.24</t>
         </is>
       </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L171" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14739,6 +14889,11 @@
           <t xml:space="preserve">14.03.24</t>
         </is>
       </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L172" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14821,6 +14976,11 @@
           <t xml:space="preserve">13.02.24</t>
         </is>
       </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L173" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14903,6 +15063,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L174" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -14985,6 +15150,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L175" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -15067,6 +15237,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L176" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -15149,6 +15324,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L177" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -15579,6 +15759,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L182" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -15661,6 +15846,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L183" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -16173,6 +16363,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L189" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -16255,6 +16450,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L190" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -16859,6 +17059,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L197" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -16941,6 +17146,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L198" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -17023,6 +17233,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L199" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -17105,6 +17320,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L200" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -17535,6 +17755,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L205" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -17617,6 +17842,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L206" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -17873,6 +18103,11 @@
           <t xml:space="preserve">30.01.24</t>
         </is>
       </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L209" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -17955,6 +18190,11 @@
           <t xml:space="preserve">30.01.24</t>
         </is>
       </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L210" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -18037,6 +18277,11 @@
           <t xml:space="preserve">30.01.24</t>
         </is>
       </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L211" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -18467,6 +18712,11 @@
           <t xml:space="preserve">26.01.24</t>
         </is>
       </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L216" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -18636,6 +18886,11 @@
           <t xml:space="preserve">28.03.24</t>
         </is>
       </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L218" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -18718,6 +18973,11 @@
           <t xml:space="preserve">28.03.24</t>
         </is>
       </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L219" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -18800,6 +19060,11 @@
           <t xml:space="preserve">28.03.24</t>
         </is>
       </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L220" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -18882,6 +19147,11 @@
           <t xml:space="preserve">28.03.24</t>
         </is>
       </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L221" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -18954,6 +19224,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L222" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19036,6 +19311,11 @@
           <t xml:space="preserve">18.03.24</t>
         </is>
       </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L223" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19118,6 +19398,11 @@
           <t xml:space="preserve">18.03.24</t>
         </is>
       </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L224" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19200,6 +19485,11 @@
           <t xml:space="preserve">18.03.24</t>
         </is>
       </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L225" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19282,6 +19572,11 @@
           <t xml:space="preserve">18.03.24</t>
         </is>
       </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L226" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19364,6 +19659,11 @@
           <t xml:space="preserve">18.03.24</t>
         </is>
       </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L227" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19446,6 +19746,11 @@
           <t xml:space="preserve">18.03.24</t>
         </is>
       </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L228" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19615,6 +19920,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L230" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19784,6 +20094,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L232" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -19866,6 +20181,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L233" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -20122,6 +20442,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L236" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -20204,6 +20529,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L237" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -20286,6 +20616,11 @@
           <t xml:space="preserve">25.01.24</t>
         </is>
       </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L238" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -20368,6 +20703,11 @@
           <t xml:space="preserve">25.01.24</t>
         </is>
       </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L239" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -21320,6 +21660,11 @@
           <t xml:space="preserve">27.11.23</t>
         </is>
       </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L250" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -21402,6 +21747,11 @@
           <t xml:space="preserve">27.11.23</t>
         </is>
       </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L251" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -23562,6 +23912,11 @@
           <t xml:space="preserve">17.07.23</t>
         </is>
       </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L276" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -23644,6 +23999,11 @@
           <t xml:space="preserve">13.07.23</t>
         </is>
       </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L277" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -25385,6 +25745,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L305" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -26530,6 +26895,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L330" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -26572,6 +26942,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L331" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -26943,6 +27318,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L339" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -26985,6 +27365,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L340" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -27074,6 +27459,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L342" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -27905,6 +28295,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L360" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -27994,6 +28389,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L362" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -28083,6 +28483,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L364" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -29149,6 +29554,11 @@
           <t xml:space="preserve">yes</t>
         </is>
       </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
+        </is>
+      </c>
       <c r="L387" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -29189,6 +29599,11 @@
       <c r="J388" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Panc1</t>
         </is>
       </c>
       <c r="L388" t="inlineStr">

</xml_diff>

<commit_message>
Add a resistance rule from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/data/neslihan.xlsx
+++ b/cellstocks/data/neslihan.xlsx
@@ -7817,7 +7817,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -9204,7 +9204,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -13114,7 +13114,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t xml:space="preserve">50CR</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -13201,7 +13201,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -13462,7 +13462,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -26136,7 +26136,7 @@
       </c>
       <c r="M312" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N312" t="inlineStr">
@@ -26606,7 +26606,7 @@
       </c>
       <c r="M322" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N322" t="inlineStr">
@@ -26935,7 +26935,7 @@
       </c>
       <c r="M329" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DtxR</t>
         </is>
       </c>
       <c r="N329" t="inlineStr">

</xml_diff>

<commit_message>
Confirm a date from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/data/neslihan.xlsx
+++ b/cellstocks/data/neslihan.xlsx
@@ -22038,14 +22038,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-01-12</t>
+        </is>
+      </c>
       <c r="I254" t="inlineStr">
         <is>
           <t xml:space="preserve">12.01.23</t>
-        </is>
-      </c>
-      <c r="J254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">

</xml_diff>

<commit_message>
Confirm 145 dates from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/data/neslihan.xlsx
+++ b/cellstocks/data/neslihan.xlsx
@@ -184,14 +184,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-01</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.24</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -271,14 +271,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-01</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.24</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -358,14 +358,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-01</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.24</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -445,14 +445,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-01</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.24</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -532,14 +532,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-01</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.24</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -619,14 +619,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-01</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.24</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1228,14 +1228,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1315,14 +1315,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1402,14 +1402,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1489,14 +1489,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1576,14 +1576,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1663,14 +1663,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1750,14 +1750,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1837,14 +1837,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1924,14 +1924,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2011,14 +2011,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2098,14 +2098,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2185,14 +2185,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2272,14 +2272,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2359,14 +2359,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2446,14 +2446,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2533,14 +2533,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2620,14 +2620,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2707,14 +2707,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-04</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t xml:space="preserve">04.01.24</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3045,14 +3045,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-09</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t xml:space="preserve">09.06.23</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3296,14 +3296,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-06</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t xml:space="preserve">06.06.23</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3470,14 +3470,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-01</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t xml:space="preserve">01.06.23</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3818,14 +3818,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-04-12</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t xml:space="preserve">12.04.23</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3900,14 +3900,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-05</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t xml:space="preserve">05.06.23</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -4248,14 +4248,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-06</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t xml:space="preserve">06.06.23</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -4509,14 +4509,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-06</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t xml:space="preserve">06.06.23</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -4596,14 +4596,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-06</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t xml:space="preserve">06.06.23</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4683,14 +4683,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -4770,14 +4770,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -4857,14 +4857,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4944,14 +4944,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -5031,14 +5031,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -5118,14 +5118,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -5205,14 +5205,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -5292,14 +5292,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -5379,14 +5379,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -5466,14 +5466,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -5553,14 +5553,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -5640,14 +5640,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -5727,14 +5727,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-07</t>
+        </is>
+      </c>
       <c r="I66" t="inlineStr">
         <is>
           <t xml:space="preserve">07.09.23</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -5814,14 +5814,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-06</t>
+        </is>
+      </c>
       <c r="I67" t="inlineStr">
         <is>
           <t xml:space="preserve">06.06.23</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -6423,14 +6423,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-02</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr">
         <is>
           <t xml:space="preserve">02.08.23</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -6597,14 +6597,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-02</t>
+        </is>
+      </c>
       <c r="I76" t="inlineStr">
         <is>
           <t xml:space="preserve">02.08.23</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -6684,14 +6684,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-02</t>
+        </is>
+      </c>
       <c r="I77" t="inlineStr">
         <is>
           <t xml:space="preserve">02.08.23</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -6771,14 +6771,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-03</t>
+        </is>
+      </c>
       <c r="I78" t="inlineStr">
         <is>
           <t xml:space="preserve">03.08.23</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -6858,14 +6858,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-03</t>
+        </is>
+      </c>
       <c r="I79" t="inlineStr">
         <is>
           <t xml:space="preserve">03.08.23</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -6945,14 +6945,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-03</t>
+        </is>
+      </c>
       <c r="I80" t="inlineStr">
         <is>
           <t xml:space="preserve">03.08.23</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -7032,14 +7032,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-03</t>
+        </is>
+      </c>
       <c r="I81" t="inlineStr">
         <is>
           <t xml:space="preserve">03.08.23</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -7119,14 +7119,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-03</t>
+        </is>
+      </c>
       <c r="I82" t="inlineStr">
         <is>
           <t xml:space="preserve">03.08.23</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -7206,14 +7206,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-09-11</t>
+        </is>
+      </c>
       <c r="I83" t="inlineStr">
         <is>
           <t xml:space="preserve">11.09.23</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -8491,14 +8491,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-10-05</t>
+        </is>
+      </c>
       <c r="I98" t="inlineStr">
         <is>
           <t xml:space="preserve">05.10.23</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -8578,14 +8578,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-10-05</t>
+        </is>
+      </c>
       <c r="I99" t="inlineStr">
         <is>
           <t xml:space="preserve">05.10.23</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -9008,14 +9008,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-10-10</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr">
         <is>
           <t xml:space="preserve">10.10.23</t>
-        </is>
-      </c>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -9095,14 +9095,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-04</t>
+        </is>
+      </c>
       <c r="I105" t="inlineStr">
         <is>
           <t xml:space="preserve">04.11.23</t>
-        </is>
-      </c>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -9182,14 +9182,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-04</t>
+        </is>
+      </c>
       <c r="I106" t="inlineStr">
         <is>
           <t xml:space="preserve">04.11.23</t>
-        </is>
-      </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -10052,14 +10052,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-03</t>
+        </is>
+      </c>
       <c r="I116" t="inlineStr">
         <is>
           <t xml:space="preserve">03.11.23</t>
-        </is>
-      </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -10308,14 +10308,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-10-10</t>
+        </is>
+      </c>
       <c r="I119" t="inlineStr">
         <is>
           <t xml:space="preserve">10.10.23</t>
-        </is>
-      </c>
-      <c r="J119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -10569,14 +10569,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-10-12</t>
+        </is>
+      </c>
       <c r="I122" t="inlineStr">
         <is>
           <t xml:space="preserve">12.10.23</t>
-        </is>
-      </c>
-      <c r="J122" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -11352,14 +11352,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-10</t>
+        </is>
+      </c>
       <c r="I131" t="inlineStr">
         <is>
           <t xml:space="preserve">10.11.23</t>
-        </is>
-      </c>
-      <c r="J131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -11439,14 +11439,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-10</t>
+        </is>
+      </c>
       <c r="I132" t="inlineStr">
         <is>
           <t xml:space="preserve">10.11.23</t>
-        </is>
-      </c>
-      <c r="J132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -11526,14 +11526,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-10</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr">
         <is>
           <t xml:space="preserve">10.11.23</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -11613,14 +11613,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-10</t>
+        </is>
+      </c>
       <c r="I134" t="inlineStr">
         <is>
           <t xml:space="preserve">10.11.23</t>
-        </is>
-      </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -11700,14 +11700,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-09</t>
+        </is>
+      </c>
       <c r="I135" t="inlineStr">
         <is>
           <t xml:space="preserve">09.11.23</t>
-        </is>
-      </c>
-      <c r="J135" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -11787,14 +11787,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-09</t>
+        </is>
+      </c>
       <c r="I136" t="inlineStr">
         <is>
           <t xml:space="preserve">09.11.23</t>
-        </is>
-      </c>
-      <c r="J136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -11874,14 +11874,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-09</t>
+        </is>
+      </c>
       <c r="I137" t="inlineStr">
         <is>
           <t xml:space="preserve">09.11.23</t>
-        </is>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -11961,14 +11961,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-07</t>
+        </is>
+      </c>
       <c r="I138" t="inlineStr">
         <is>
           <t xml:space="preserve">07.11.23</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -12048,14 +12048,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-07</t>
+        </is>
+      </c>
       <c r="I139" t="inlineStr">
         <is>
           <t xml:space="preserve">07.11.23</t>
-        </is>
-      </c>
-      <c r="J139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -12396,14 +12396,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-12-01</t>
+        </is>
+      </c>
       <c r="I143" t="inlineStr">
         <is>
           <t xml:space="preserve">01.12.23</t>
-        </is>
-      </c>
-      <c r="J143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -12483,14 +12483,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-12-04</t>
+        </is>
+      </c>
       <c r="I144" t="inlineStr">
         <is>
           <t xml:space="preserve">04.12.23</t>
-        </is>
-      </c>
-      <c r="J144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -12570,14 +12570,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-12-08</t>
+        </is>
+      </c>
       <c r="I145" t="inlineStr">
         <is>
           <t xml:space="preserve">08.12.23</t>
-        </is>
-      </c>
-      <c r="J145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -12744,14 +12744,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-12-08</t>
+        </is>
+      </c>
       <c r="I147" t="inlineStr">
         <is>
           <t xml:space="preserve">08.12.23</t>
-        </is>
-      </c>
-      <c r="J147" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -12918,14 +12918,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-08-11</t>
+        </is>
+      </c>
       <c r="I149" t="inlineStr">
         <is>
           <t xml:space="preserve">11.08.23</t>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -13092,14 +13092,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-04-05</t>
+        </is>
+      </c>
       <c r="I151" t="inlineStr">
         <is>
           <t xml:space="preserve">05.04.24</t>
-        </is>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -13179,14 +13179,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-04-05</t>
+        </is>
+      </c>
       <c r="I152" t="inlineStr">
         <is>
           <t xml:space="preserve">05.04.24</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -13266,14 +13266,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-04-08</t>
+        </is>
+      </c>
       <c r="I153" t="inlineStr">
         <is>
           <t xml:space="preserve">08.04.23</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -13353,14 +13353,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-04-08</t>
+        </is>
+      </c>
       <c r="I154" t="inlineStr">
         <is>
           <t xml:space="preserve">08.04.23</t>
-        </is>
-      </c>
-      <c r="J154" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -13440,14 +13440,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-04-05</t>
+        </is>
+      </c>
       <c r="I155" t="inlineStr">
         <is>
           <t xml:space="preserve">05.04.24</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -13527,14 +13527,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-03-04</t>
+        </is>
+      </c>
       <c r="I156" t="inlineStr">
         <is>
           <t xml:space="preserve">04.03.24</t>
-        </is>
-      </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -13614,14 +13614,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-03-04</t>
+        </is>
+      </c>
       <c r="I157" t="inlineStr">
         <is>
           <t xml:space="preserve">04.03.24</t>
-        </is>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -13701,14 +13701,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-03-04</t>
+        </is>
+      </c>
       <c r="I158" t="inlineStr">
         <is>
           <t xml:space="preserve">04.03.24</t>
-        </is>
-      </c>
-      <c r="J158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -13788,14 +13788,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-03-04</t>
+        </is>
+      </c>
       <c r="I159" t="inlineStr">
         <is>
           <t xml:space="preserve">04.03.24</t>
-        </is>
-      </c>
-      <c r="J159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -13875,14 +13875,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-03-04</t>
+        </is>
+      </c>
       <c r="I160" t="inlineStr">
         <is>
           <t xml:space="preserve">04.03.24</t>
-        </is>
-      </c>
-      <c r="J160" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -13962,14 +13962,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-03-04</t>
+        </is>
+      </c>
       <c r="I161" t="inlineStr">
         <is>
           <t xml:space="preserve">04.03.24</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -15093,14 +15093,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I174" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J174" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -15180,14 +15180,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I175" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J175" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -15267,14 +15267,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I176" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J176" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -15354,14 +15354,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I177" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J177" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -15441,14 +15441,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I178" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -15528,14 +15528,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I179" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J179" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -15615,14 +15615,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I180" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J180" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -15702,14 +15702,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I181" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J181" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -15789,14 +15789,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I182" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J182" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -15876,14 +15876,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I183" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J183" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -15963,14 +15963,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I184" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J184" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -16050,14 +16050,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I185" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J185" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -16137,14 +16137,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I186" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J186" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -16224,14 +16224,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I187" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J187" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -16306,14 +16306,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-09</t>
+        </is>
+      </c>
       <c r="I188" t="inlineStr">
         <is>
           <t xml:space="preserve">09.02.24</t>
-        </is>
-      </c>
-      <c r="J188" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -16393,14 +16393,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-08</t>
+        </is>
+      </c>
       <c r="I189" t="inlineStr">
         <is>
           <t xml:space="preserve">08.02.24</t>
-        </is>
-      </c>
-      <c r="J189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -16480,14 +16480,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-08</t>
+        </is>
+      </c>
       <c r="I190" t="inlineStr">
         <is>
           <t xml:space="preserve">08.02.24</t>
-        </is>
-      </c>
-      <c r="J190" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -16567,14 +16567,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-08</t>
+        </is>
+      </c>
       <c r="I191" t="inlineStr">
         <is>
           <t xml:space="preserve">08.02.24</t>
-        </is>
-      </c>
-      <c r="J191" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -16654,14 +16654,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-08</t>
+        </is>
+      </c>
       <c r="I192" t="inlineStr">
         <is>
           <t xml:space="preserve">08.02.24</t>
-        </is>
-      </c>
-      <c r="J192" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -16741,14 +16741,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-06</t>
+        </is>
+      </c>
       <c r="I193" t="inlineStr">
         <is>
           <t xml:space="preserve">06.02.24</t>
-        </is>
-      </c>
-      <c r="J193" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -16828,14 +16828,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-06</t>
+        </is>
+      </c>
       <c r="I194" t="inlineStr">
         <is>
           <t xml:space="preserve">06.02.24</t>
-        </is>
-      </c>
-      <c r="J194" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -16915,14 +16915,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-06</t>
+        </is>
+      </c>
       <c r="I195" t="inlineStr">
         <is>
           <t xml:space="preserve">06.02.24</t>
-        </is>
-      </c>
-      <c r="J195" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -17002,14 +17002,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-06</t>
+        </is>
+      </c>
       <c r="I196" t="inlineStr">
         <is>
           <t xml:space="preserve">06.02.24</t>
-        </is>
-      </c>
-      <c r="J196" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -17089,14 +17089,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-03</t>
+        </is>
+      </c>
       <c r="I197" t="inlineStr">
         <is>
           <t xml:space="preserve">03.02.24</t>
-        </is>
-      </c>
-      <c r="J197" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -17176,14 +17176,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-03</t>
+        </is>
+      </c>
       <c r="I198" t="inlineStr">
         <is>
           <t xml:space="preserve">03.02.24</t>
-        </is>
-      </c>
-      <c r="J198" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -17263,14 +17263,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-03</t>
+        </is>
+      </c>
       <c r="I199" t="inlineStr">
         <is>
           <t xml:space="preserve">03.02.24</t>
-        </is>
-      </c>
-      <c r="J199" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -17350,14 +17350,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-03</t>
+        </is>
+      </c>
       <c r="I200" t="inlineStr">
         <is>
           <t xml:space="preserve">03.02.24</t>
-        </is>
-      </c>
-      <c r="J200" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -17437,14 +17437,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-02</t>
+        </is>
+      </c>
       <c r="I201" t="inlineStr">
         <is>
           <t xml:space="preserve">02.02.24</t>
-        </is>
-      </c>
-      <c r="J201" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -17524,14 +17524,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-02</t>
+        </is>
+      </c>
       <c r="I202" t="inlineStr">
         <is>
           <t xml:space="preserve">02.02.24</t>
-        </is>
-      </c>
-      <c r="J202" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -17611,14 +17611,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-02</t>
+        </is>
+      </c>
       <c r="I203" t="inlineStr">
         <is>
           <t xml:space="preserve">02.02.24</t>
-        </is>
-      </c>
-      <c r="J203" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -17698,14 +17698,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-02</t>
+        </is>
+      </c>
       <c r="I204" t="inlineStr">
         <is>
           <t xml:space="preserve">02.02.24</t>
-        </is>
-      </c>
-      <c r="J204" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -17785,14 +17785,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-02</t>
+        </is>
+      </c>
       <c r="I205" t="inlineStr">
         <is>
           <t xml:space="preserve">02.02.24</t>
-        </is>
-      </c>
-      <c r="J205" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -17872,14 +17872,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-02</t>
+        </is>
+      </c>
       <c r="I206" t="inlineStr">
         <is>
           <t xml:space="preserve">02.02.24</t>
-        </is>
-      </c>
-      <c r="J206" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -17959,14 +17959,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-02</t>
+        </is>
+      </c>
       <c r="I207" t="inlineStr">
         <is>
           <t xml:space="preserve">02.02.24</t>
-        </is>
-      </c>
-      <c r="J207" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -18046,14 +18046,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-02-02</t>
+        </is>
+      </c>
       <c r="I208" t="inlineStr">
         <is>
           <t xml:space="preserve">02.02.24</t>
-        </is>
-      </c>
-      <c r="J208" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -19950,14 +19950,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-12</t>
+        </is>
+      </c>
       <c r="I230" t="inlineStr">
         <is>
           <t xml:space="preserve">12.01.24</t>
-        </is>
-      </c>
-      <c r="J230" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -20037,14 +20037,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-09</t>
+        </is>
+      </c>
       <c r="I231" t="inlineStr">
         <is>
           <t xml:space="preserve">09.01.24</t>
-        </is>
-      </c>
-      <c r="J231" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -20124,14 +20124,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-09</t>
+        </is>
+      </c>
       <c r="I232" t="inlineStr">
         <is>
           <t xml:space="preserve">09.01.24</t>
-        </is>
-      </c>
-      <c r="J232" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -20211,14 +20211,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-09</t>
+        </is>
+      </c>
       <c r="I233" t="inlineStr">
         <is>
           <t xml:space="preserve">09.01.24</t>
-        </is>
-      </c>
-      <c r="J233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -20298,14 +20298,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-09</t>
+        </is>
+      </c>
       <c r="I234" t="inlineStr">
         <is>
           <t xml:space="preserve">09.01.24</t>
-        </is>
-      </c>
-      <c r="J234" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -20385,14 +20385,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-09</t>
+        </is>
+      </c>
       <c r="I235" t="inlineStr">
         <is>
           <t xml:space="preserve">09.01.24</t>
-        </is>
-      </c>
-      <c r="J235" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -20472,14 +20472,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-09</t>
+        </is>
+      </c>
       <c r="I236" t="inlineStr">
         <is>
           <t xml:space="preserve">09.01.24</t>
-        </is>
-      </c>
-      <c r="J236" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -20559,14 +20559,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-12</t>
+        </is>
+      </c>
       <c r="I237" t="inlineStr">
         <is>
           <t xml:space="preserve">12.01.24</t>
-        </is>
-      </c>
-      <c r="J237" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -20907,14 +20907,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-07-10</t>
+        </is>
+      </c>
       <c r="I241" t="inlineStr">
         <is>
           <t xml:space="preserve">10.07.23</t>
-        </is>
-      </c>
-      <c r="J241" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -21081,14 +21081,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-07-03</t>
+        </is>
+      </c>
       <c r="I243" t="inlineStr">
         <is>
           <t xml:space="preserve">03.07.23</t>
-        </is>
-      </c>
-      <c r="J243" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -21255,14 +21255,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-05</t>
+        </is>
+      </c>
       <c r="I245" t="inlineStr">
         <is>
           <t xml:space="preserve">05.06.23</t>
-        </is>
-      </c>
-      <c r="J245" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -21429,14 +21429,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-03</t>
+        </is>
+      </c>
       <c r="I247" t="inlineStr">
         <is>
           <t xml:space="preserve">03.06.23</t>
-        </is>
-      </c>
-      <c r="J247" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -22125,14 +22125,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2022-12-09</t>
+        </is>
+      </c>
       <c r="I255" t="inlineStr">
         <is>
           <t xml:space="preserve">09.12.22</t>
-        </is>
-      </c>
-      <c r="J255" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -22299,14 +22299,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-01-06</t>
+        </is>
+      </c>
       <c r="I257" t="inlineStr">
         <is>
           <t xml:space="preserve">06.01.23</t>
-        </is>
-      </c>
-      <c r="J257" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -22386,14 +22386,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-04-05</t>
+        </is>
+      </c>
       <c r="I258" t="inlineStr">
         <is>
           <t xml:space="preserve">05.04.23</t>
-        </is>
-      </c>
-      <c r="J258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -22821,14 +22821,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-04-04</t>
+        </is>
+      </c>
       <c r="I263" t="inlineStr">
         <is>
           <t xml:space="preserve">04.04.23</t>
-        </is>
-      </c>
-      <c r="J263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -23256,14 +23256,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-04-11</t>
+        </is>
+      </c>
       <c r="I268" t="inlineStr">
         <is>
           <t xml:space="preserve">11.04.23</t>
-        </is>
-      </c>
-      <c r="J268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -24213,14 +24213,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-07-10</t>
+        </is>
+      </c>
       <c r="I279" t="inlineStr">
         <is>
           <t xml:space="preserve">10.07.23</t>
-        </is>
-      </c>
-      <c r="J279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -24474,14 +24474,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-07-11</t>
+        </is>
+      </c>
       <c r="I282" t="inlineStr">
         <is>
           <t xml:space="preserve">11.07.23</t>
-        </is>
-      </c>
-      <c r="J282" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -24648,14 +24648,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-09</t>
+        </is>
+      </c>
       <c r="I284" t="inlineStr">
         <is>
           <t xml:space="preserve">09.06.23</t>
-        </is>
-      </c>
-      <c r="J284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -24822,14 +24822,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-01</t>
+        </is>
+      </c>
       <c r="I286" t="inlineStr">
         <is>
           <t xml:space="preserve">01.06.23</t>
-        </is>
-      </c>
-      <c r="J286" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -24996,14 +24996,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-06-09</t>
+        </is>
+      </c>
       <c r="I288" t="inlineStr">
         <is>
           <t xml:space="preserve">09.06.23</t>
-        </is>
-      </c>
-      <c r="J288" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K288" t="inlineStr">

</xml_diff>